<commit_message>
Implementacion de Asistente de Restauracion, advertencia por perdida de datos, validacion de ultimo administrador activo y semillas de traduccion
</commit_message>
<xml_diff>
--- a/Documentacion/Plan Entrega IS y TD 2026.xlsx
+++ b/Documentacion/Plan Entrega IS y TD 2026.xlsx
@@ -1,15 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1273D646-486C-472F-A45F-14ED43610EF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42BA0112-2889-4AB1-AEF5-82D4244E0AC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" tabRatio="699" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="699" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan Entregas IS 2026" sheetId="2" r:id="rId1"/>
-    <sheet name="Cronograma" sheetId="8" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -32,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="59">
   <si>
     <t>Iteración</t>
   </si>
@@ -209,46 +208,13 @@
   </si>
   <si>
     <t>De, al menos, los cambios realizados durante el ciclo de vida de alguna entidad. Se entiende que esta funcionalidad responde al concepto de auditoria y se espera que el sistema permita realizar  una trazabilidad detallada sobre todos los cambios realizados en la entidad elegida. De esta manera responde a "quién?", "cuándo?" y "qué?" proponiendo un historial y con la posibilidad de recomponer el estado anterior de un objeto determinado</t>
-  </si>
-  <si>
-    <t>Clase</t>
-  </si>
-  <si>
-    <t>Fecha</t>
-  </si>
-  <si>
-    <t>Tema</t>
-  </si>
-  <si>
-    <t>Introducción</t>
-  </si>
-  <si>
-    <t>Recuperatorio</t>
-  </si>
-  <si>
-    <t>Entrega 1</t>
-  </si>
-  <si>
-    <t>Parcial 1</t>
-  </si>
-  <si>
-    <t>Entrega 2</t>
-  </si>
-  <si>
-    <t>Parcial 2</t>
-  </si>
-  <si>
-    <t>Entrega 3</t>
-  </si>
-  <si>
-    <t>FERIADO</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -264,15 +230,8 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="6">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -291,18 +250,6 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="-0.249977111117893"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="27">
     <border>
@@ -654,7 +601,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -708,13 +655,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="16" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="16" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="16" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1074,23 +1014,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E27"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="64.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="103.7109375" customWidth="1"/>
-    <col min="5" max="5" width="66.28515625" style="13" customWidth="1"/>
+    <col min="3" max="3" width="64.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="103.6640625" customWidth="1"/>
+    <col min="5" max="5" width="66.33203125" style="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="26" t="s">
+    <row r="1" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="19" t="s">
         <v>57</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-    </row>
-    <row r="2" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+    </row>
+    <row r="2" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -1107,8 +1047,8 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="75.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="36">
+    <row r="3" spans="1:5" ht="58.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="29">
         <v>1</v>
       </c>
       <c r="B3" s="15"/>
@@ -1122,8 +1062,8 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="105.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="36"/>
+    <row r="4" spans="1:5" ht="101.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="29"/>
       <c r="B4" s="15"/>
       <c r="C4" s="14" t="s">
         <v>8</v>
@@ -1135,8 +1075,8 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="105.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="36"/>
+    <row r="5" spans="1:5" ht="87" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="29"/>
       <c r="B5" s="15"/>
       <c r="C5" s="2" t="s">
         <v>11</v>
@@ -1148,8 +1088,8 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="105.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="36"/>
+    <row r="6" spans="1:5" ht="87" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="29"/>
       <c r="B6" s="15"/>
       <c r="C6" s="14" t="s">
         <v>14</v>
@@ -1161,8 +1101,8 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="41">
+    <row r="7" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="34">
         <v>2</v>
       </c>
       <c r="B7" s="15"/>
@@ -1176,8 +1116,8 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="270.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="42"/>
+    <row r="8" spans="1:5" ht="231" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="35"/>
       <c r="B8" s="15"/>
       <c r="C8" s="3" t="s">
         <v>19</v>
@@ -1189,8 +1129,8 @@
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="42"/>
+    <row r="9" spans="1:5" ht="58.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="35"/>
       <c r="B9" s="15"/>
       <c r="C9" s="14" t="s">
         <v>21</v>
@@ -1202,8 +1142,8 @@
         <v>23</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="75.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="42"/>
+    <row r="10" spans="1:5" ht="58.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="35"/>
       <c r="B10" s="15"/>
       <c r="C10" s="14" t="s">
         <v>24</v>
@@ -1213,8 +1153,8 @@
       </c>
       <c r="E10" s="14"/>
     </row>
-    <row r="11" spans="1:5" ht="90.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="43"/>
+    <row r="11" spans="1:5" ht="87" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="36"/>
       <c r="B11" s="15"/>
       <c r="C11" s="14" t="s">
         <v>25</v>
@@ -1226,8 +1166,8 @@
         <v>27</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="37">
+    <row r="12" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="30">
         <v>3</v>
       </c>
       <c r="B12" s="15"/>
@@ -1241,8 +1181,8 @@
         <v>23</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="36"/>
+    <row r="13" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="29"/>
       <c r="B13" s="15"/>
       <c r="C13" s="3" t="s">
         <v>29</v>
@@ -1254,8 +1194,8 @@
         <v>13</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="36"/>
+    <row r="14" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="29"/>
       <c r="B14" s="15"/>
       <c r="C14" s="14" t="s">
         <v>25</v>
@@ -1267,8 +1207,8 @@
         <v>27</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="36"/>
+    <row r="15" spans="1:5" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="29"/>
       <c r="B15" s="15"/>
       <c r="C15" s="14" t="s">
         <v>30</v>
@@ -1280,8 +1220,8 @@
         <v>32</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="38"/>
+    <row r="16" spans="1:5" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="31"/>
       <c r="B16" s="15"/>
       <c r="C16" s="14" t="s">
         <v>33</v>
@@ -1293,87 +1233,87 @@
         <v>35</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="32" t="s">
+    <row r="17" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="25" t="s">
         <v>36</v>
       </c>
-      <c r="B17" s="32"/>
-      <c r="C17" s="32"/>
-      <c r="D17" s="32"/>
-    </row>
-    <row r="18" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="B17" s="25"/>
+      <c r="C17" s="25"/>
+      <c r="D17" s="25"/>
+    </row>
+    <row r="18" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A18" s="8">
         <v>1</v>
       </c>
-      <c r="B18" s="33" t="s">
+      <c r="B18" s="26" t="s">
         <v>37</v>
       </c>
-      <c r="C18" s="34"/>
+      <c r="C18" s="27"/>
       <c r="D18" s="4" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" s="9">
         <v>2</v>
       </c>
-      <c r="B19" s="39" t="s">
+      <c r="B19" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="C19" s="40"/>
+      <c r="C19" s="33"/>
       <c r="D19" s="5" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" s="10">
         <v>3</v>
       </c>
-      <c r="B20" s="29" t="s">
+      <c r="B20" s="22" t="s">
         <v>41</v>
       </c>
-      <c r="C20" s="35"/>
+      <c r="C20" s="28"/>
       <c r="D20" s="6" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" s="10">
         <v>4</v>
       </c>
-      <c r="B21" s="28" t="s">
+      <c r="B21" s="21" t="s">
         <v>43</v>
       </c>
-      <c r="C21" s="29"/>
+      <c r="C21" s="22"/>
       <c r="D21" s="6" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" s="10">
         <v>5</v>
       </c>
-      <c r="B22" s="28" t="s">
+      <c r="B22" s="21" t="s">
         <v>45</v>
       </c>
-      <c r="C22" s="29"/>
+      <c r="C22" s="22"/>
       <c r="D22" s="6" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" s="10">
         <v>6</v>
       </c>
-      <c r="B23" s="28" t="s">
+      <c r="B23" s="21" t="s">
         <v>47</v>
       </c>
-      <c r="C23" s="29"/>
+      <c r="C23" s="22"/>
       <c r="D23" s="6" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" s="10">
         <v>6</v>
       </c>
@@ -1385,38 +1325,38 @@
         <v>50</v>
       </c>
     </row>
-    <row r="25" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" s="10">
         <v>7</v>
       </c>
-      <c r="B25" s="28" t="s">
+      <c r="B25" s="21" t="s">
         <v>51</v>
       </c>
-      <c r="C25" s="29"/>
+      <c r="C25" s="22"/>
       <c r="D25" s="6" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="26" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A26" s="10">
         <v>8</v>
       </c>
-      <c r="B26" s="28" t="s">
+      <c r="B26" s="21" t="s">
         <v>53</v>
       </c>
-      <c r="C26" s="29"/>
+      <c r="C26" s="22"/>
       <c r="D26" s="6" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="27" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A27" s="11">
         <v>9</v>
       </c>
-      <c r="B27" s="30" t="s">
+      <c r="B27" s="23" t="s">
         <v>55</v>
       </c>
-      <c r="C27" s="31"/>
+      <c r="C27" s="24"/>
       <c r="D27" s="7" t="s">
         <v>56</v>
       </c>
@@ -1441,172 +1381,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F854E2D-0B73-46F0-A47C-EC8E21F4946D}">
-  <dimension ref="A1:C16"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="3" max="3" width="13.5703125" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>59</v>
-      </c>
-      <c r="B1" t="s">
-        <v>60</v>
-      </c>
-      <c r="C1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2" s="19">
-        <v>46121</v>
-      </c>
-      <c r="C2" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3" s="19">
-        <v>46128</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4" s="19">
-        <v>46135</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="24">
-        <v>4</v>
-      </c>
-      <c r="B5" s="25">
-        <v>46142</v>
-      </c>
-      <c r="C5" s="24" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6">
-        <v>5</v>
-      </c>
-      <c r="B6" s="19">
-        <v>46149</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7">
-        <v>6</v>
-      </c>
-      <c r="B7" s="19">
-        <v>46156</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="22">
-        <v>7</v>
-      </c>
-      <c r="B8" s="23">
-        <v>46163</v>
-      </c>
-      <c r="C8" s="22" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9">
-        <v>8</v>
-      </c>
-      <c r="B9" s="19">
-        <v>46170</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10">
-        <v>9</v>
-      </c>
-      <c r="B10" s="19">
-        <v>46177</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="24">
-        <v>10</v>
-      </c>
-      <c r="B11" s="25">
-        <v>46184</v>
-      </c>
-      <c r="C11" s="24" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12">
-        <v>11</v>
-      </c>
-      <c r="B12" s="19">
-        <v>46191</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="22">
-        <v>12</v>
-      </c>
-      <c r="B13" s="23">
-        <v>46198</v>
-      </c>
-      <c r="C13" s="22" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="24">
-        <v>13</v>
-      </c>
-      <c r="B14" s="25">
-        <v>46205</v>
-      </c>
-      <c r="C14" s="24" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" s="20">
-        <v>14</v>
-      </c>
-      <c r="B15" s="21">
-        <v>46212</v>
-      </c>
-      <c r="C15" s="20" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" s="22">
-        <v>15</v>
-      </c>
-      <c r="B16" s="23">
-        <v>46219</v>
-      </c>
-      <c r="C16" s="22" t="s">
-        <v>63</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>